<commit_message>
Corrige dependencias e configuracao de execucao
</commit_message>
<xml_diff>
--- a/resultado.xlsx
+++ b/resultado.xlsx
@@ -431,12 +431,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
@@ -476,16 +476,16 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>13/01</t>
+          <t>10/06</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Lançamentos:compras esaques 13/01 99APP *99AppSaoP 15,03</t>
+          <t>10/06 99APP *99AppSao P 11,80</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>15.03</v>
+        <v>11.8</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -499,16 +499,16 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>13/01</t>
+          <t>12/06</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>13/01 99APP *99AppSaoP 15,20</t>
+          <t>12/06 99APP *99AppSao P 12,60</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>15.2</v>
+        <v>12.6</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -522,16 +522,16 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>21/01</t>
+          <t>16/06</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>21/01 99APP *99AppSaoP 7,12</t>
+          <t>16/06 99APP *99AppSao P 9,80</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>7.12</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E4" t="n">
         <v>2</v>
@@ -540,21 +540,21 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>UBER*</t>
+          <t>99APP *</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>23/01</t>
+          <t>17/06</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>23/01 UberUBER*TRIPHELP.US 33,71</t>
+          <t>17/06 99APP *99AppSao P 9,67</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>33.71</v>
+        <v>9.67</v>
       </c>
       <c r="E5" t="n">
         <v>2</v>
@@ -563,21 +563,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>UBER*</t>
+          <t>99APP *</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>23/01</t>
+          <t>19/06</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>23/01 DL *Uber*RidesSaoP 46,95</t>
+          <t>19/06 99APP *99AppSao P 13,90</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>46.95</v>
+        <v>13.9</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -591,16 +591,16 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>26/01</t>
+          <t>02/06</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>26/01 99APP *99AppSaoP 10,20</t>
+          <t>02/06 99APP *99AppSao P 9,50</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>10.2</v>
+        <v>9.5</v>
       </c>
       <c r="E7" t="n">
         <v>2</v>
@@ -614,16 +614,16 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>27/01</t>
+          <t>23/06</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>27/01 99APP *99AppSaoP 11,30</t>
+          <t>23/06 99APP *99AppSao P 10,20</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>11.3</v>
+        <v>10.2</v>
       </c>
       <c r="E8" t="n">
         <v>2</v>
@@ -637,18 +637,64 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>30/01</t>
+          <t>03/06</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>30/01 99APP *99AppSaoP 12,40</t>
+          <t>03/06 99APP *99AppSao P 13,80</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>12.4</v>
+        <v>13.8</v>
       </c>
       <c r="E9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>99APP *</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>05/06</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>05/06 99APP *99AppSao P 12,80</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>99APP *</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>26/06</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>26/06 99APP *99AppSao P 11,70</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="E11" t="n">
         <v>2</v>
       </c>
     </row>
@@ -689,7 +735,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>80.66</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -699,7 +745,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>71.25</v>
+        <v>115.77</v>
       </c>
     </row>
     <row r="4">
@@ -709,7 +755,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>151.91</v>
+        <v>115.77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>